<commit_message>
0.8.4 ground and tact polishing
+ добавил арту в битву на тактическом уровнье
</commit_message>
<xml_diff>
--- a/player_brigade.xlsx
+++ b/player_brigade.xlsx
@@ -2716,7 +2716,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M50" t="n">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M51" t="n">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M53" t="n">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M55" t="n">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M56" t="n">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M57" t="n">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M59" t="n">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P59" t="n">
         <v>0</v>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M60" t="n">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M61" t="n">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M62" t="n">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M63" t="n">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M64" t="n">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M65" t="n">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M67" t="n">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M68" t="n">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M69" t="n">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M70" t="n">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M71" t="n">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M72" t="n">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M73" t="n">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M110" t="n">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P110" t="n">
         <v>0</v>
@@ -7096,7 +7096,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M111" t="n">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="N113" t="inlineStr"/>
       <c r="O113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P113" t="n">
         <v>0</v>
@@ -7276,7 +7276,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>died_from_injury</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M114" t="n">
@@ -7456,7 +7456,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M117" t="n">
@@ -7516,7 +7516,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M118" t="n">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="N118" t="inlineStr"/>
       <c r="O118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P118" t="n">
         <v>0</v>
@@ -7584,7 +7584,7 @@
       </c>
       <c r="N119" t="inlineStr"/>
       <c r="O119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P119" t="n">
         <v>0</v>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M121" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="N122" t="inlineStr"/>
       <c r="O122" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P122" t="n">
         <v>0</v>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M123" t="n">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="N124" t="inlineStr"/>
       <c r="O124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P124" t="n">
         <v>0</v>
@@ -7996,7 +7996,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M126" t="n">
@@ -8124,7 +8124,7 @@
       </c>
       <c r="N128" t="inlineStr"/>
       <c r="O128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P128" t="n">
         <v>0</v>
@@ -8184,7 +8184,7 @@
       </c>
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P129" t="n">
         <v>0</v>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M130" t="n">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="N130" t="inlineStr"/>
       <c r="O130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P130" t="n">
         <v>0</v>
@@ -8296,7 +8296,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M131" t="n">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M132" t="n">
@@ -8416,7 +8416,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M133" t="n">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="N135" t="inlineStr"/>
       <c r="O135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P135" t="n">
         <v>0</v>
@@ -8596,7 +8596,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M136" t="n">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="N136" t="inlineStr"/>
       <c r="O136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P136" t="n">
         <v>0</v>
@@ -8656,7 +8656,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M137" t="n">
@@ -8836,7 +8836,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M140" t="n">
@@ -8844,7 +8844,7 @@
       </c>
       <c r="N140" t="inlineStr"/>
       <c r="O140" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P140" t="n">
         <v>0</v>
@@ -8896,7 +8896,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M141" t="n">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M142" t="n">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M146" t="n">
@@ -9256,7 +9256,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M147" t="n">
@@ -9316,7 +9316,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M148" t="n">
@@ -9384,7 +9384,7 @@
       </c>
       <c r="N149" t="inlineStr"/>
       <c r="O149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P149" t="n">
         <v>0</v>
@@ -9496,7 +9496,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M151" t="n">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M152" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="N152" t="inlineStr"/>
       <c r="O152" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P152" t="n">
         <v>0</v>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M153" t="n">
@@ -9624,7 +9624,7 @@
       </c>
       <c r="N153" t="inlineStr"/>
       <c r="O153" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P153" t="n">
         <v>0</v>
@@ -9676,7 +9676,7 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M154" t="n">
@@ -9684,7 +9684,7 @@
       </c>
       <c r="N154" t="inlineStr"/>
       <c r="O154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P154" t="n">
         <v>0</v>
@@ -9796,7 +9796,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M156" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="N157" t="inlineStr"/>
       <c r="O157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P157" t="n">
         <v>0</v>
@@ -9976,7 +9976,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M159" t="n">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M160" t="n">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="N161" t="inlineStr"/>
       <c r="O161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P161" t="n">
         <v>0</v>
@@ -10156,7 +10156,7 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M162" t="n">
@@ -10336,7 +10336,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M165" t="n">
@@ -10396,7 +10396,7 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M166" t="n">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M168" t="n">
@@ -10524,7 +10524,7 @@
       </c>
       <c r="N168" t="inlineStr"/>
       <c r="O168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P168" t="n">
         <v>0</v>
@@ -10876,7 +10876,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M174" t="n">
@@ -10936,7 +10936,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M175" t="n">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M176" t="n">
@@ -11296,7 +11296,7 @@
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M181" t="n">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M182" t="n">
@@ -11476,7 +11476,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M184" t="n">
@@ -11596,7 +11596,7 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M186" t="n">
@@ -11656,7 +11656,7 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M187" t="n">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M188" t="n">
@@ -11776,7 +11776,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M189" t="n">
@@ -11836,7 +11836,7 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M190" t="n">
@@ -12016,7 +12016,7 @@
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M193" t="n">
@@ -12024,7 +12024,7 @@
       </c>
       <c r="N193" t="inlineStr"/>
       <c r="O193" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P193" t="n">
         <v>0</v>
@@ -12076,7 +12076,7 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M194" t="n">
@@ -12196,7 +12196,7 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M196" t="n">
@@ -12204,7 +12204,7 @@
       </c>
       <c r="N196" t="inlineStr"/>
       <c r="O196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P196" t="n">
         <v>0</v>
@@ -12376,7 +12376,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M199" t="n">
@@ -12384,7 +12384,7 @@
       </c>
       <c r="N199" t="inlineStr"/>
       <c r="O199" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P199" t="n">
         <v>0</v>
@@ -12436,7 +12436,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M200" t="n">
@@ -12496,7 +12496,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M201" t="n">
@@ -12676,7 +12676,7 @@
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M204" t="n">
@@ -12736,7 +12736,7 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M205" t="n">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M206" t="n">
@@ -12916,7 +12916,7 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M208" t="n">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="N208" t="inlineStr"/>
       <c r="O208" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P208" t="n">
         <v>0</v>
@@ -12976,7 +12976,7 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M209" t="n">
@@ -13156,7 +13156,7 @@
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M212" t="n">
@@ -13164,7 +13164,7 @@
       </c>
       <c r="N212" t="inlineStr"/>
       <c r="O212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P212" t="n">
         <v>0</v>
@@ -13276,7 +13276,7 @@
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M214" t="n">
@@ -13284,7 +13284,7 @@
       </c>
       <c r="N214" t="inlineStr"/>
       <c r="O214" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P214" t="n">
         <v>0</v>
@@ -13336,7 +13336,7 @@
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M215" t="n">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M216" t="n">
@@ -13644,7 +13644,7 @@
       </c>
       <c r="N220" t="inlineStr"/>
       <c r="O220" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P220" t="n">
         <v>0</v>
@@ -13756,7 +13756,7 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M222" t="n">
@@ -14004,7 +14004,7 @@
       </c>
       <c r="N226" t="inlineStr"/>
       <c r="O226" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P226" t="n">
         <v>0</v>
@@ -14176,7 +14176,7 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M229" t="n">
@@ -14296,7 +14296,7 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M231" t="n">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="N235" t="inlineStr"/>
       <c r="O235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P235" t="n">
         <v>0</v>
@@ -14604,7 +14604,7 @@
       </c>
       <c r="N236" t="inlineStr"/>
       <c r="O236" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P236" t="n">
         <v>0</v>
@@ -15016,7 +15016,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M243" t="n">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="N243" t="inlineStr"/>
       <c r="O243" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P243" t="n">
         <v>0</v>
@@ -15144,7 +15144,7 @@
       </c>
       <c r="N245" t="inlineStr"/>
       <c r="O245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P245" t="n">
         <v>0</v>
@@ -15196,7 +15196,7 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>died_from_injury</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M246" t="n">
@@ -15264,7 +15264,7 @@
       </c>
       <c r="N247" t="inlineStr"/>
       <c r="O247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P247" t="n">
         <v>0</v>
@@ -15384,7 +15384,7 @@
       </c>
       <c r="N249" t="inlineStr"/>
       <c r="O249" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P249" t="n">
         <v>0</v>
@@ -15556,7 +15556,7 @@
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M252" t="n">
@@ -15564,7 +15564,7 @@
       </c>
       <c r="N252" t="inlineStr"/>
       <c r="O252" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P252" t="n">
         <v>0</v>
@@ -15736,7 +15736,7 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M255" t="n">
@@ -16456,7 +16456,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M267" t="n">
@@ -16816,7 +16816,7 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M273" t="n">
@@ -16996,7 +16996,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M276" t="n">
@@ -17116,7 +17116,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M278" t="n">
@@ -17896,7 +17896,7 @@
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M291" t="n">
@@ -18084,7 +18084,7 @@
       </c>
       <c r="N294" t="inlineStr"/>
       <c r="O294" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P294" t="n">
         <v>0</v>
@@ -18196,7 +18196,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M296" t="n">
@@ -18204,7 +18204,7 @@
       </c>
       <c r="N296" t="inlineStr"/>
       <c r="O296" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P296" t="n">
         <v>0</v>
@@ -18256,7 +18256,7 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M297" t="n">
@@ -18264,7 +18264,7 @@
       </c>
       <c r="N297" t="inlineStr"/>
       <c r="O297" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P297" t="n">
         <v>0</v>
@@ -18384,7 +18384,7 @@
       </c>
       <c r="N299" t="inlineStr"/>
       <c r="O299" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P299" t="n">
         <v>0</v>
@@ -18496,7 +18496,7 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M301" t="n">
@@ -18564,7 +18564,7 @@
       </c>
       <c r="N302" t="inlineStr"/>
       <c r="O302" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P302" t="n">
         <v>0</v>
@@ -18624,7 +18624,7 @@
       </c>
       <c r="N303" t="inlineStr"/>
       <c r="O303" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P303" t="n">
         <v>0</v>
@@ -18796,7 +18796,7 @@
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M306" t="n">
@@ -18804,7 +18804,7 @@
       </c>
       <c r="N306" t="inlineStr"/>
       <c r="O306" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P306" t="n">
         <v>0</v>
@@ -18924,7 +18924,7 @@
       </c>
       <c r="N308" t="inlineStr"/>
       <c r="O308" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P308" t="n">
         <v>0</v>
@@ -18976,7 +18976,7 @@
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>died_from_injury</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M309" t="n">
@@ -19164,7 +19164,7 @@
       </c>
       <c r="N312" t="inlineStr"/>
       <c r="O312" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P312" t="n">
         <v>0</v>
@@ -19224,7 +19224,7 @@
       </c>
       <c r="N313" t="inlineStr"/>
       <c r="O313" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P313" t="n">
         <v>0</v>
@@ -19276,7 +19276,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M314" t="n">
@@ -19284,7 +19284,7 @@
       </c>
       <c r="N314" t="inlineStr"/>
       <c r="O314" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P314" t="n">
         <v>0</v>
@@ -19344,7 +19344,7 @@
       </c>
       <c r="N315" t="inlineStr"/>
       <c r="O315" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P315" t="n">
         <v>0</v>
@@ -19584,7 +19584,7 @@
       </c>
       <c r="N319" t="inlineStr"/>
       <c r="O319" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P319" t="n">
         <v>0</v>
@@ -19876,7 +19876,7 @@
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M324" t="n">
@@ -19884,7 +19884,7 @@
       </c>
       <c r="N324" t="inlineStr"/>
       <c r="O324" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P324" t="n">
         <v>0</v>
@@ -19944,7 +19944,7 @@
       </c>
       <c r="N325" t="inlineStr"/>
       <c r="O325" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P325" t="n">
         <v>0</v>

</xml_diff>